<commit_message>
Implementar flujo operacional del conductor en Mobile
- Implementa listado y detalle de servicios asignados al conductor
- Agrega inicio de servicio con validaciones del Backend
- Muestra estado e inicio real en horario de Chile
- Integra visualización del QR activo sin regenerar el token
- Agrega consulta de pasajeros y estados de asistencia
- Incorpora resumen de asistencia y pasajeros planificados/no planificados
- Agrega navegación, estados de carga, errores y pull-to-refresh
- Mantiene rutas protegidas para el rol CONDUCTOR
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Gantt CAPSTONE - SISTEMA DE GESTION PARA TRANSPORTE DE PASAJEROS.xlsx
+++ b/FASE 1/Evidencias Grupales/Gantt CAPSTONE - SISTEMA DE GESTION PARA TRANSPORTE DE PASAJEROS.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\capstone-2026\FASE 1\Evidencias Grupales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32D5B373-F735-4516-A216-8CD2DEB8FD36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{500733D6-3ECF-4E6A-B5DE-32ADB553163D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gestión Proyecto Carta Gantt" sheetId="3" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gestión Proyecto Carta Gantt'!$D$1:$D$45</definedName>
+  </definedNames>
   <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -1512,6 +1515,30 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="20" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1530,12 +1557,6 @@
     <xf numFmtId="0" fontId="4" fillId="10" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1545,12 +1566,6 @@
     <xf numFmtId="0" fontId="4" fillId="14" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1560,12 +1575,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1573,12 +1582,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="22" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1897,86 +1900,86 @@
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
-      <c r="I7" s="84"/>
-      <c r="J7" s="85"/>
-      <c r="K7" s="85"/>
-      <c r="L7" s="85"/>
-      <c r="M7" s="85"/>
-      <c r="N7" s="85"/>
-      <c r="O7" s="85"/>
-      <c r="P7" s="85"/>
-      <c r="Q7" s="85"/>
-      <c r="R7" s="85"/>
-      <c r="S7" s="85"/>
-      <c r="T7" s="85"/>
-      <c r="U7" s="85"/>
-      <c r="V7" s="85"/>
-      <c r="W7" s="85"/>
-      <c r="X7" s="85"/>
-      <c r="Y7" s="85"/>
-      <c r="Z7" s="85"/>
-      <c r="AA7" s="85"/>
-      <c r="AB7" s="86"/>
-      <c r="AC7" s="89"/>
-      <c r="AD7" s="90"/>
-      <c r="AE7" s="90"/>
-      <c r="AF7" s="90"/>
-      <c r="AG7" s="90"/>
-      <c r="AH7" s="90"/>
-      <c r="AI7" s="90"/>
-      <c r="AJ7" s="90"/>
-      <c r="AK7" s="90"/>
-      <c r="AL7" s="90"/>
-      <c r="AM7" s="90"/>
-      <c r="AN7" s="90"/>
-      <c r="AO7" s="90"/>
-      <c r="AP7" s="90"/>
-      <c r="AQ7" s="90"/>
-      <c r="AR7" s="90"/>
-      <c r="AS7" s="90"/>
-      <c r="AT7" s="90"/>
-      <c r="AU7" s="90"/>
-      <c r="AV7" s="91"/>
-      <c r="AW7" s="94"/>
-      <c r="AX7" s="95"/>
-      <c r="AY7" s="95"/>
-      <c r="AZ7" s="95"/>
-      <c r="BA7" s="95"/>
-      <c r="BB7" s="95"/>
-      <c r="BC7" s="95"/>
-      <c r="BD7" s="95"/>
-      <c r="BE7" s="95"/>
-      <c r="BF7" s="95"/>
-      <c r="BG7" s="95"/>
-      <c r="BH7" s="95"/>
-      <c r="BI7" s="95"/>
-      <c r="BJ7" s="95"/>
-      <c r="BK7" s="95"/>
-      <c r="BL7" s="95"/>
-      <c r="BM7" s="95"/>
-      <c r="BN7" s="95"/>
-      <c r="BO7" s="95"/>
-      <c r="BP7" s="96"/>
-      <c r="BQ7" s="99"/>
-      <c r="BR7" s="100"/>
-      <c r="BS7" s="100"/>
-      <c r="BT7" s="100"/>
-      <c r="BU7" s="100"/>
-      <c r="BV7" s="100"/>
-      <c r="BW7" s="100"/>
-      <c r="BX7" s="100"/>
-      <c r="BY7" s="100"/>
-      <c r="BZ7" s="100"/>
-      <c r="CA7" s="100"/>
-      <c r="CB7" s="100"/>
-      <c r="CC7" s="100"/>
-      <c r="CD7" s="100"/>
-      <c r="CE7" s="100"/>
-      <c r="CF7" s="100"/>
-      <c r="CG7" s="100"/>
-      <c r="CH7" s="100"/>
-      <c r="CI7" s="100"/>
-      <c r="CJ7" s="101"/>
+      <c r="I7" s="92"/>
+      <c r="J7" s="93"/>
+      <c r="K7" s="93"/>
+      <c r="L7" s="93"/>
+      <c r="M7" s="93"/>
+      <c r="N7" s="93"/>
+      <c r="O7" s="93"/>
+      <c r="P7" s="93"/>
+      <c r="Q7" s="93"/>
+      <c r="R7" s="93"/>
+      <c r="S7" s="93"/>
+      <c r="T7" s="93"/>
+      <c r="U7" s="93"/>
+      <c r="V7" s="93"/>
+      <c r="W7" s="93"/>
+      <c r="X7" s="93"/>
+      <c r="Y7" s="93"/>
+      <c r="Z7" s="93"/>
+      <c r="AA7" s="93"/>
+      <c r="AB7" s="94"/>
+      <c r="AC7" s="95"/>
+      <c r="AD7" s="96"/>
+      <c r="AE7" s="96"/>
+      <c r="AF7" s="96"/>
+      <c r="AG7" s="96"/>
+      <c r="AH7" s="96"/>
+      <c r="AI7" s="96"/>
+      <c r="AJ7" s="96"/>
+      <c r="AK7" s="96"/>
+      <c r="AL7" s="96"/>
+      <c r="AM7" s="96"/>
+      <c r="AN7" s="96"/>
+      <c r="AO7" s="96"/>
+      <c r="AP7" s="96"/>
+      <c r="AQ7" s="96"/>
+      <c r="AR7" s="96"/>
+      <c r="AS7" s="96"/>
+      <c r="AT7" s="96"/>
+      <c r="AU7" s="96"/>
+      <c r="AV7" s="97"/>
+      <c r="AW7" s="98"/>
+      <c r="AX7" s="99"/>
+      <c r="AY7" s="99"/>
+      <c r="AZ7" s="99"/>
+      <c r="BA7" s="99"/>
+      <c r="BB7" s="99"/>
+      <c r="BC7" s="99"/>
+      <c r="BD7" s="99"/>
+      <c r="BE7" s="99"/>
+      <c r="BF7" s="99"/>
+      <c r="BG7" s="99"/>
+      <c r="BH7" s="99"/>
+      <c r="BI7" s="99"/>
+      <c r="BJ7" s="99"/>
+      <c r="BK7" s="99"/>
+      <c r="BL7" s="99"/>
+      <c r="BM7" s="99"/>
+      <c r="BN7" s="99"/>
+      <c r="BO7" s="99"/>
+      <c r="BP7" s="100"/>
+      <c r="BQ7" s="101"/>
+      <c r="BR7" s="102"/>
+      <c r="BS7" s="102"/>
+      <c r="BT7" s="102"/>
+      <c r="BU7" s="102"/>
+      <c r="BV7" s="102"/>
+      <c r="BW7" s="102"/>
+      <c r="BX7" s="102"/>
+      <c r="BY7" s="102"/>
+      <c r="BZ7" s="102"/>
+      <c r="CA7" s="102"/>
+      <c r="CB7" s="102"/>
+      <c r="CC7" s="102"/>
+      <c r="CD7" s="102"/>
+      <c r="CE7" s="102"/>
+      <c r="CF7" s="102"/>
+      <c r="CG7" s="102"/>
+      <c r="CH7" s="102"/>
+      <c r="CI7" s="102"/>
+      <c r="CJ7" s="103"/>
       <c r="CK7" s="104" t="s">
         <v>52</v>
       </c>
@@ -2008,111 +2011,111 @@
       <c r="H8" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="87" t="s">
+      <c r="I8" s="83" t="s">
         <v>30</v>
       </c>
-      <c r="J8" s="88"/>
-      <c r="K8" s="88"/>
-      <c r="L8" s="88"/>
-      <c r="M8" s="88"/>
-      <c r="N8" s="87" t="s">
+      <c r="J8" s="84"/>
+      <c r="K8" s="84"/>
+      <c r="L8" s="84"/>
+      <c r="M8" s="84"/>
+      <c r="N8" s="83" t="s">
         <v>31</v>
       </c>
-      <c r="O8" s="88"/>
-      <c r="P8" s="88"/>
-      <c r="Q8" s="88"/>
-      <c r="R8" s="88"/>
-      <c r="S8" s="87" t="s">
+      <c r="O8" s="84"/>
+      <c r="P8" s="84"/>
+      <c r="Q8" s="84"/>
+      <c r="R8" s="84"/>
+      <c r="S8" s="83" t="s">
         <v>32</v>
       </c>
-      <c r="T8" s="88"/>
-      <c r="U8" s="88"/>
-      <c r="V8" s="88"/>
-      <c r="W8" s="88"/>
-      <c r="X8" s="87" t="s">
+      <c r="T8" s="84"/>
+      <c r="U8" s="84"/>
+      <c r="V8" s="84"/>
+      <c r="W8" s="84"/>
+      <c r="X8" s="83" t="s">
         <v>33</v>
       </c>
-      <c r="Y8" s="88"/>
-      <c r="Z8" s="88"/>
-      <c r="AA8" s="88"/>
-      <c r="AB8" s="88"/>
-      <c r="AC8" s="92" t="s">
+      <c r="Y8" s="84"/>
+      <c r="Z8" s="84"/>
+      <c r="AA8" s="84"/>
+      <c r="AB8" s="84"/>
+      <c r="AC8" s="85" t="s">
         <v>34</v>
       </c>
-      <c r="AD8" s="93"/>
-      <c r="AE8" s="93"/>
-      <c r="AF8" s="93"/>
-      <c r="AG8" s="93"/>
-      <c r="AH8" s="92" t="s">
+      <c r="AD8" s="86"/>
+      <c r="AE8" s="86"/>
+      <c r="AF8" s="86"/>
+      <c r="AG8" s="86"/>
+      <c r="AH8" s="85" t="s">
         <v>35</v>
       </c>
-      <c r="AI8" s="93"/>
-      <c r="AJ8" s="93"/>
-      <c r="AK8" s="93"/>
-      <c r="AL8" s="93"/>
-      <c r="AM8" s="92" t="s">
+      <c r="AI8" s="86"/>
+      <c r="AJ8" s="86"/>
+      <c r="AK8" s="86"/>
+      <c r="AL8" s="86"/>
+      <c r="AM8" s="85" t="s">
         <v>36</v>
       </c>
-      <c r="AN8" s="93"/>
-      <c r="AO8" s="93"/>
-      <c r="AP8" s="93"/>
-      <c r="AQ8" s="93"/>
-      <c r="AR8" s="92" t="s">
+      <c r="AN8" s="86"/>
+      <c r="AO8" s="86"/>
+      <c r="AP8" s="86"/>
+      <c r="AQ8" s="86"/>
+      <c r="AR8" s="85" t="s">
         <v>37</v>
       </c>
-      <c r="AS8" s="93"/>
-      <c r="AT8" s="93"/>
-      <c r="AU8" s="93"/>
-      <c r="AV8" s="93"/>
-      <c r="AW8" s="97" t="s">
+      <c r="AS8" s="86"/>
+      <c r="AT8" s="86"/>
+      <c r="AU8" s="86"/>
+      <c r="AV8" s="86"/>
+      <c r="AW8" s="87" t="s">
         <v>38</v>
       </c>
-      <c r="AX8" s="98"/>
-      <c r="AY8" s="98"/>
-      <c r="AZ8" s="98"/>
-      <c r="BA8" s="98"/>
-      <c r="BB8" s="97" t="s">
+      <c r="AX8" s="88"/>
+      <c r="AY8" s="88"/>
+      <c r="AZ8" s="88"/>
+      <c r="BA8" s="88"/>
+      <c r="BB8" s="87" t="s">
         <v>39</v>
       </c>
-      <c r="BC8" s="98"/>
-      <c r="BD8" s="98"/>
-      <c r="BE8" s="98"/>
-      <c r="BF8" s="98"/>
-      <c r="BG8" s="97" t="s">
+      <c r="BC8" s="88"/>
+      <c r="BD8" s="88"/>
+      <c r="BE8" s="88"/>
+      <c r="BF8" s="88"/>
+      <c r="BG8" s="87" t="s">
         <v>40</v>
       </c>
-      <c r="BH8" s="98"/>
-      <c r="BI8" s="98"/>
-      <c r="BJ8" s="98"/>
-      <c r="BK8" s="98"/>
-      <c r="BL8" s="97" t="s">
+      <c r="BH8" s="88"/>
+      <c r="BI8" s="88"/>
+      <c r="BJ8" s="88"/>
+      <c r="BK8" s="88"/>
+      <c r="BL8" s="87" t="s">
         <v>41</v>
       </c>
-      <c r="BM8" s="98"/>
-      <c r="BN8" s="98"/>
-      <c r="BO8" s="98"/>
-      <c r="BP8" s="98"/>
-      <c r="BQ8" s="102" t="s">
+      <c r="BM8" s="88"/>
+      <c r="BN8" s="88"/>
+      <c r="BO8" s="88"/>
+      <c r="BP8" s="88"/>
+      <c r="BQ8" s="81" t="s">
         <v>47</v>
       </c>
-      <c r="BR8" s="103"/>
-      <c r="BS8" s="103"/>
-      <c r="BT8" s="103"/>
-      <c r="BU8" s="103"/>
-      <c r="BV8" s="102" t="s">
+      <c r="BR8" s="82"/>
+      <c r="BS8" s="82"/>
+      <c r="BT8" s="82"/>
+      <c r="BU8" s="82"/>
+      <c r="BV8" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="BW8" s="103"/>
-      <c r="BX8" s="103"/>
-      <c r="BY8" s="103"/>
-      <c r="BZ8" s="103"/>
-      <c r="CA8" s="102" t="s">
+      <c r="BW8" s="82"/>
+      <c r="BX8" s="82"/>
+      <c r="BY8" s="82"/>
+      <c r="BZ8" s="82"/>
+      <c r="CA8" s="81" t="s">
         <v>49</v>
       </c>
-      <c r="CB8" s="103"/>
-      <c r="CC8" s="103"/>
-      <c r="CD8" s="103"/>
-      <c r="CE8" s="103"/>
+      <c r="CB8" s="82"/>
+      <c r="CC8" s="82"/>
+      <c r="CD8" s="82"/>
+      <c r="CE8" s="82"/>
       <c r="CF8" s="106" t="s">
         <v>50</v>
       </c>
@@ -2120,13 +2123,13 @@
       <c r="CH8" s="107"/>
       <c r="CI8" s="107"/>
       <c r="CJ8" s="108"/>
-      <c r="CK8" s="81" t="s">
+      <c r="CK8" s="89" t="s">
         <v>51</v>
       </c>
-      <c r="CL8" s="82"/>
-      <c r="CM8" s="82"/>
-      <c r="CN8" s="82"/>
-      <c r="CO8" s="83"/>
+      <c r="CL8" s="90"/>
+      <c r="CM8" s="90"/>
+      <c r="CN8" s="90"/>
+      <c r="CO8" s="91"/>
       <c r="CP8" s="57"/>
     </row>
     <row r="9" spans="2:94" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6349,13 +6352,8 @@
       <c r="C45" s="3"/>
     </row>
   </sheetData>
+  <autoFilter ref="D1:D45" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <mergeCells count="22">
-    <mergeCell ref="BV8:BZ8"/>
-    <mergeCell ref="S8:W8"/>
-    <mergeCell ref="AC8:AG8"/>
-    <mergeCell ref="AH8:AL8"/>
-    <mergeCell ref="AR8:AV8"/>
-    <mergeCell ref="AW8:BA8"/>
     <mergeCell ref="CK8:CO8"/>
     <mergeCell ref="I7:AB7"/>
     <mergeCell ref="X8:AB8"/>
@@ -6372,6 +6370,12 @@
     <mergeCell ref="BB8:BF8"/>
     <mergeCell ref="BL8:BP8"/>
     <mergeCell ref="BQ8:BU8"/>
+    <mergeCell ref="BV8:BZ8"/>
+    <mergeCell ref="S8:W8"/>
+    <mergeCell ref="AC8:AG8"/>
+    <mergeCell ref="AH8:AL8"/>
+    <mergeCell ref="AR8:AV8"/>
+    <mergeCell ref="AW8:BA8"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <conditionalFormatting sqref="D37:G37">

</xml_diff>